<commit_message>
vault backup: 2026-05-31 17:49:35
</commit_message>
<xml_diff>
--- a/BWL/Übung/Übungen/UE08/ue08.xlsx
+++ b/BWL/Übung/Übungen/UE08/ue08.xlsx
@@ -16,7 +16,13 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+  <si>
+    <t>a)</t>
+  </si>
+  <si>
+    <t>b)</t>
+  </si>
   <si>
     <t>Fixkosten</t>
   </si>
@@ -94,12 +100,12 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:w="http://schemas.openxmlformats.org/wordprocessingml/2006/main">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>314203</xdr:colOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>199902</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>87629</xdr:rowOff>
+      <xdr:rowOff>87628</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="5615108" cy="2459354"/>
+    <xdr:ext cx="5615107" cy="2459353"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="812829405" name=""/>
@@ -113,7 +119,7 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm flipH="0" flipV="0">
-          <a:off x="1533403" y="262889"/>
+          <a:off x="809502" y="262888"/>
           <a:ext cx="5615108" cy="2459354"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -616,44 +622,57 @@
     <row r="8" ht="14.25">
       <c r="I8" s="1"/>
     </row>
-    <row r="19" ht="14.25">
-      <c r="D19" t="s">
+    <row r="18" ht="14.25">
+      <c r="B18" t="s">
         <v>0</v>
       </c>
-      <c r="E19" t="s">
+    </row>
+    <row r="20" ht="14.25">
+      <c r="G20"/>
+    </row>
+    <row r="32" ht="14.25">
+      <c r="B32" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="20" ht="14.25">
-      <c r="C20" t="s">
+    <row r="33" ht="14.25">
+      <c r="D33" t="s">
         <v>2</v>
       </c>
-      <c r="D20">
+      <c r="E33" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34" ht="14.25">
+      <c r="C34" t="s">
+        <v>4</v>
+      </c>
+      <c r="D34">
         <v>80000</v>
       </c>
     </row>
-    <row r="21" ht="14.25">
-      <c r="C21" t="s">
-        <v>3</v>
-      </c>
-      <c r="D21">
+    <row r="35" ht="14.25">
+      <c r="C35" t="s">
+        <v>5</v>
+      </c>
+      <c r="D35">
         <v>160000</v>
       </c>
     </row>
-    <row r="22" ht="14.25">
-      <c r="C22" t="s">
-        <v>4</v>
-      </c>
-      <c r="D22">
-        <f>SUM(D20:D21)</f>
+    <row r="36" ht="14.25">
+      <c r="C36" t="s">
+        <v>6</v>
+      </c>
+      <c r="D36">
+        <f>SUM(D34:D35)</f>
         <v>240000</v>
       </c>
     </row>
-    <row r="24" ht="14.25">
-      <c r="C24" t="s">
-        <v>5</v>
-      </c>
-      <c r="D24">
+    <row r="38" ht="14.25">
+      <c r="C38" t="s">
+        <v>7</v>
+      </c>
+      <c r="D38">
         <f>480000/98*100</f>
         <v>489795.91836734687</v>
       </c>

</xml_diff>

<commit_message>
vault backup: 2026-06-01 19:54:51
</commit_message>
<xml_diff>
--- a/BWL/Übung/Übungen/UE08/ue08.xlsx
+++ b/BWL/Übung/Übungen/UE08/ue08.xlsx
@@ -16,36 +16,94 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t>a)</t>
   </si>
   <si>
+    <t>Umsatz</t>
+  </si>
+  <si>
+    <t>Wareneinsatz</t>
+  </si>
+  <si>
+    <t>Provision</t>
+  </si>
+  <si>
+    <t>Deckungsbeitrag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deckungsbeitrag muss genau gleich Fixkosten werden</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d.h. 0.48 * Umsatz = 240k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">240.000 / 0.48 =</t>
+  </si>
+  <si>
     <t>b)</t>
   </si>
   <si>
-    <t>Fixkosten</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Variable Kosten</t>
-  </si>
-  <si>
-    <t>Gehälter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">zusätz. Fixkosten</t>
-  </si>
-  <si>
-    <t>Gesamtfixkosten</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Umsatz muss also </t>
+    <t xml:space="preserve">Betriebsergebnis * 100 / Umsatz = 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Betriebsergebnis: Umsatzerlöse - var. Kosten  - Fixkosten</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Betriebsergebnis soll also 4 % des Umsatzes ausmachen, also:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BE = 0,04 * Umsatz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">db_Gesamt - Fixkosten = Betriebsergebnis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">also: 0,48*Umsatz-Fixkosten=0,04*Umsatz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/ - 0,04*Umsatz / + Fixkosten</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,44*Umsatz = Fixkosten</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,44*Umsatz = 240k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">erforderlicher Umsatz:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Umsatz = 240k / 0,44 = </t>
+  </si>
+  <si>
+    <t>c)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wareneinsatz: Aufschlag = 120 %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100 / 2,2 = </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deckungsbeitrag (Umsatz - Prov - Einsatz)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Umsatz bei 300.000€ wäre also 300.000 * 2,2 =</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Betriebsergebnis wäre dann 660000 * 0,5255 - Fixkosten</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$€-407]_-;\-* #,##0.00\ [$€-407]_-;_-* &quot;-&quot;??\ [$€-407]_-;_-@_-"/>
+    <numFmt numFmtId="165" formatCode="#,##0.00\ [$€-407]"/>
+  </numFmts>
   <fonts count="1">
     <font>
       <sz val="11.000000"/>
@@ -54,12 +112,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="5"/>
+        <bgColor indexed="5"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -74,11 +138,19 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="8">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="10" xfId="0" applyNumberFormat="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf fontId="0" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFill="1"/>
+    <xf fontId="0" fillId="2" borderId="0" numFmtId="164" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="10" xfId="0" applyNumberFormat="1">
+      <protection hidden="0" locked="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="165" xfId="0" applyNumberFormat="1"/>
+    <xf fontId="0" fillId="2" borderId="0" numFmtId="165" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -94,42 +166,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:w="http://schemas.openxmlformats.org/wordprocessingml/2006/main">
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>199902</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>87628</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="5615107" cy="2459353"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="812829405" name=""/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill rotWithShape="1">
-        <a:blip r:embed="rId1"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm flipH="0" flipV="0">
-          <a:off x="809502" y="262888"/>
-          <a:ext cx="5615108" cy="2459354"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme.xml><?xml version="1.0" encoding="utf-8"?>
@@ -612,76 +648,216 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="1"/>
+  </sheetPr>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col customWidth="1" min="3" max="3" width="19.28125"/>
-    <col customWidth="1" min="4" max="4" width="14.8515625"/>
+    <col bestFit="1" min="2" max="2" width="53.203125"/>
+    <col customWidth="1" min="3" max="3" width="11.00390625"/>
+    <col bestFit="1" customWidth="1" min="4" max="4" width="20.0625"/>
     <col customWidth="1" min="5" max="5" width="17.28125"/>
   </cols>
   <sheetData>
+    <row r="1" ht="14.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" ht="14.25">
+      <c r="B2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" ht="14.25">
+      <c r="B3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="1">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="4" ht="14.25">
+      <c r="B4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" s="1">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="5" ht="14.25">
+      <c r="B5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="1">
+        <v>0.47999999999999998</v>
+      </c>
+    </row>
+    <row r="7" ht="14.25">
+      <c r="B7" t="s">
+        <v>5</v>
+      </c>
+    </row>
     <row r="8" ht="14.25">
-      <c r="I8" s="1"/>
+      <c r="B8" t="s">
+        <v>6</v>
+      </c>
+      <c r="I8" s="2"/>
+    </row>
+    <row r="9" ht="14.25">
+      <c r="B9" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9" s="3">
+        <f>240000/0.48</f>
+        <v>500000</v>
+      </c>
+    </row>
+    <row r="14" ht="14.25">
+      <c r="A14" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15" ht="14.25">
+      <c r="B15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" ht="14.25">
+      <c r="B16" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="18" ht="14.25">
       <c r="B18" t="s">
-        <v>0</v>
+        <v>11</v>
       </c>
     </row>
     <row r="20" ht="14.25">
-      <c r="G20"/>
+      <c r="B20" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="24" ht="14.25">
+      <c r="B24" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="25" ht="14.25">
+      <c r="B25" t="s">
+        <v>14</v>
+      </c>
+      <c r="C25" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="26" ht="14.25">
+      <c r="B26" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="27" ht="14.25">
+      <c r="B27" t="s">
+        <v>17</v>
+      </c>
+      <c r="D27" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="28" ht="14.25">
+      <c r="B28" t="s">
+        <v>19</v>
+      </c>
+      <c r="D28" s="4">
+        <f>240000/0.44</f>
+        <v>545454.54545454541</v>
+      </c>
     </row>
     <row r="32" ht="14.25">
+      <c r="A32" t="s">
+        <v>20</v>
+      </c>
       <c r="B32" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="34" ht="14.25">
+      <c r="B34" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="33" ht="14.25">
-      <c r="D33" t="s">
+      <c r="C34" s="1">
+        <v>1</v>
+      </c>
+      <c r="E34" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="35" ht="14.25">
+      <c r="B35" t="s">
+        <v>3</v>
+      </c>
+      <c r="C35" s="1">
+        <v>0.02</v>
+      </c>
+      <c r="E35" t="s">
+        <v>22</v>
+      </c>
+      <c r="F35">
+        <f>100/2.2</f>
+        <v>45.454545454545453</v>
+      </c>
+    </row>
+    <row r="36" ht="14.25">
+      <c r="B36" t="s">
         <v>2</v>
       </c>
-      <c r="E33" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="34" ht="14.25">
-      <c r="C34" t="s">
-        <v>4</v>
-      </c>
-      <c r="D34">
-        <v>80000</v>
-      </c>
-    </row>
-    <row r="35" ht="14.25">
-      <c r="C35" t="s">
-        <v>5</v>
-      </c>
-      <c r="D35">
-        <v>160000</v>
-      </c>
-    </row>
-    <row r="36" ht="14.25">
-      <c r="C36" t="s">
-        <v>6</v>
-      </c>
-      <c r="D36">
-        <f>SUM(D34:D35)</f>
-        <v>240000</v>
+      <c r="C36" s="5">
+        <f>100/2.2/100</f>
+        <v>0.45454545454545453</v>
+      </c>
+    </row>
+    <row r="37" ht="14.25">
+      <c r="B37" t="s">
+        <v>23</v>
+      </c>
+      <c r="C37" s="1">
+        <f>C34-C35-C36</f>
+        <v>0.5254545454545454</v>
       </c>
     </row>
     <row r="38" ht="14.25">
-      <c r="C38" t="s">
-        <v>7</v>
-      </c>
-      <c r="D38">
-        <f>480000/98*100</f>
-        <v>489795.91836734687</v>
+      <c r="C38" s="1"/>
+    </row>
+    <row r="39" ht="14.25">
+      <c r="C39" s="1"/>
+    </row>
+    <row r="40" ht="14.25">
+      <c r="B40" t="s">
+        <v>24</v>
+      </c>
+      <c r="C40" s="1"/>
+      <c r="D40" s="6">
+        <f>300000*2.2</f>
+        <v>660000</v>
+      </c>
+    </row>
+    <row r="41" ht="14.25">
+      <c r="B41" t="s">
+        <v>25</v>
+      </c>
+      <c r="D41" s="7">
+        <f>D40*C37-240000</f>
+        <v>106799.99999999994</v>
       </c>
     </row>
   </sheetData>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <pageSetup paperSize="9" scale="85" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
   <headerFooter/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
vault backup: 2026-06-08 17:28:41
</commit_message>
<xml_diff>
--- a/BWL/Übung/Übungen/UE08/ue08.xlsx
+++ b/BWL/Übung/Übungen/UE08/ue08.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
     <t>a)</t>
   </si>
@@ -37,6 +37,9 @@
   </si>
   <si>
     <t xml:space="preserve">d.h. 0.48 * Umsatz = 240k</t>
+  </si>
+  <si>
+    <t>K_f/(p-K_v)</t>
   </si>
   <si>
     <t xml:space="preserve">240.000 / 0.48 =</t>
@@ -706,11 +709,14 @@
       <c r="B8" t="s">
         <v>6</v>
       </c>
+      <c r="E8" t="s">
+        <v>7</v>
+      </c>
       <c r="I8" s="2"/>
     </row>
     <row r="9" ht="14.25">
       <c r="B9" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C9" s="3">
         <f>240000/0.48</f>
@@ -719,58 +725,58 @@
     </row>
     <row r="14" ht="14.25">
       <c r="A14" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="15" ht="14.25">
       <c r="B15" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16" ht="14.25">
       <c r="B16" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="18" ht="14.25">
       <c r="B18" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="20" ht="14.25">
       <c r="B20" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="24" ht="14.25">
       <c r="B24" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="25" ht="14.25">
       <c r="B25" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C25" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="26" ht="14.25">
       <c r="B26" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="27" ht="14.25">
       <c r="B27" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D27" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="28" ht="14.25">
       <c r="B28" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D28" s="4">
         <f>240000/0.44</f>
@@ -779,10 +785,10 @@
     </row>
     <row r="32" ht="14.25">
       <c r="A32" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B32" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="34" ht="14.25">
@@ -793,7 +799,7 @@
         <v>1</v>
       </c>
       <c r="E34" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="35" ht="14.25">
@@ -804,7 +810,7 @@
         <v>0.02</v>
       </c>
       <c r="E35" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F35">
         <f>100/2.2</f>
@@ -822,7 +828,7 @@
     </row>
     <row r="37" ht="14.25">
       <c r="B37" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C37" s="1">
         <f>C34-C35-C36</f>
@@ -837,7 +843,7 @@
     </row>
     <row r="40" ht="14.25">
       <c r="B40" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C40" s="1"/>
       <c r="D40" s="6">
@@ -847,7 +853,7 @@
     </row>
     <row r="41" ht="14.25">
       <c r="B41" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D41" s="7">
         <f>D40*C37-240000</f>

</xml_diff>